<commit_message>
feat(F-NAR-019): ATOM-EMO.LEX.003-03 Victorina et le bac à sable
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.LEX.003-03.xlsx
+++ b/stories/arbres/ATOM-EMO.LEX.003-03.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>parc, aiguilles de pin</t>
+          <t>parc, aiguilles de pin, bac, sable, balançoire, pelle, seau, pin, manche</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Au parc, les balançoires sont prises. Victorina dit qu'elle est déçue. Elle cherche une autre idée. Elle creuse au bac à sable.</t>
+          <t>Victorina connaît le parc. Les aiguilles de pin craquent. Sur le manche, un éclat de pelle luit. Elle veut la balançoire, maintenant. Les balançoires sont prises. Sourire parti. Poitrine trop vite. Papa s'accroupit. Elle dit je suis déçue. Elle va au bac. Elle creuse. Merci vécu. Deuxième ruse : bac occupé, pelle coincée. Elle refuse de foncer. Un éclat de pelle tient sur le manche.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Des aiguilles de pin sont sur le chemin. Elles piquent un peu sous les chaussures. Un seau jaune attend près du sable. Une sonnette de vélo tinte, plus loin. Le toboggan est froid sous la main. Ça sent le pin, tout doux. Je range le sac près des pins. On reste ensemble, d'accord ? D'accord, papa. Tu as vu le seau jaune ? Oui. Il attend. En ce moment, Victorina veut la balançoire. La chaîne brille un peu. Celle-là, papa. On regarde, oui. Les deux balançoires bougent déjà. Il n'y a plus de place. Elles sont prises... Victorina sent une boule. Ses épaules tombent un peu. Je suis déçue. Tu es déçue. Ce n'est pas honteux. Un souhait peut attendre. On nomme. On cherche une autre idée. Souffle une fois, Victorina. Victorina souffle. Elle regarde le seau jaune. Le bac à sable, alors. Le bac. C'est une autre idée. Bravo. Tu as nommé : déçue. Ils vont au bac. Le sable est frais et un peu lourd. Victorina creuse. Le seau jaune se remplit. Un tas, papa. Un tas, oui. Tu veux un autre seau ? Celui-là. Le jaune. La déception diminue. Être déçue, ce n'est pas honteux. Une autre idée peut venir. Le bac, alors. Oui. Le bac. Les aiguilles de pin restent sur le chemin. La sonnette tinte encore, plus loin.</t>
+          <t>Victorina connaît le parc, ses odeurs, ses bruits. Je le connais, papa. Tu le connais, le parc ? Oui, papa. Les aiguilles de pin craquent sous les chaussures. Elles craquent, maman. Tu les entends, les aiguilles ? Oui, maman. Ça sent le pin, un peu tiède. Ça sent le pin. Tu le sens, le pin ? Oui, papa. Une pelle rouge attend près du bac. Elle est rouge ! Tu la vois, la pelle ? Oui, maman. Sur le manche, un éclat de pelle luit. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Un seau jaune repose contre le sable. Le seau est jaune. Il attend, près du bac. Oui. Les chaînes des balançoires cliquettent, plus loin. Je les entends. Elles bougent, Victorina ? Oui, maman. Un détail paraît nouveau, sur le manche. Le point clair. Tu le regardes, Victorina ? Oui, papa. En ce moment, Victorina veut la balançoire. Je veux celle-là, maintenant ! Tout de suite ? Oui, papa. Victorina court trop vite vers les chaînes. Les deux balançoires bougent, occupées. Il n'y a plus de place. Elles sont prises. Le sourire de Victorina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Sa poitrine va trop vite. Oh. Elles sont prises, Victorina ? Oui, papa. Tes épaules tombent, Victorina ? Un peu, maman. L'éclat de pelle tremble, puis tient. Papa s'accroupit à la même hauteur, sans parler. Je suis déçue. Tu as une boule, Victorina ? Oui, papa. Ses épaules restent basses, près des chaînes. Elle tourne la tête vers le bac.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Des aiguilles de pin sont sur le chemin. Elles piquent un peu sous les chaussures. Un seau jaune attend près du sable. Une sonnette de vélo tinte, plus loin. Le toboggan est froid sous la main. Ça sent le pin, tout doux. Je range le sac près des pins. On reste ensemble, d'accord ? D'accord, papa. Tu as vu le seau jaune ? Oui. Il attend. En ce moment, Victorina veut la balançoire. La chaîne brille un peu. Celle-là, papa. On regarde, oui. Les deux balançoires bougent déjà. Il n'y a plus de place. Elles sont prises... Victorina sent une boule. Ses épaules tombent un peu. Je suis déçue. Tu es déçue. Ce n'est pas honteux. Un souhait peut attendre. On nomme. On cherche une autre idée. Souffle une fois, Victorina. Victorina souffle. Elle regarde le seau jaune. Le bac à sable, alors. Le bac. C'est une autre idée. Bravo. Tu as nommé : déçue. Ils vont au bac. Le sable est frais et un peu lourd. Victorina creuse. Le seau jaune se remplit. Un tas, papa. Un tas, oui. Tu veux un autre seau ? Celui-là. Le jaune. La déception diminue. Être déçue, ce n'est pas honteux. Une autre idée peut venir. Le bac, alors. Oui. Le bac. Les aiguilles de pin restent sur le chemin. La sonnette tinte encore, plus loin.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorina connaît le parc, ses odeurs, ses bruits. Je le connais, papa. Tu le connais, le parc ? Oui, papa. Les aiguilles de pin craquent sous les chaussures. Elles craquent, maman. Tu les entends, les aiguilles ? Oui, maman. Ça sent le pin, un peu tiède. Ça sent le pin. Tu le sens, le pin ? Oui, papa. Une pelle rouge attend près du bac. Elle est rouge ! Tu la vois, la pelle ? Oui, maman. Sur le manche, un &lt;emphasis level="moderate"&gt;éclat de pelle&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Un seau jaune repose contre le sable. Le seau est jaune. Il attend, près du bac. Oui. Les chaînes des balançoires cliquettent, plus loin. Je les entends. Elles bougent, Victorina ? Oui, maman. Un détail paraît nouveau, sur le manche. Le point clair. Tu le regardes, Victorina ? Oui, papa. En ce moment, Victorina veut la balançoire. Je veux celle-là, maintenant ! Tout de suite ? Oui, papa. Victorina court trop vite vers les chaînes. Les deux balançoires bougent, occupées. Il n'y a plus de place. Elles sont prises. Le sourire de Victorina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Sa poitrine va trop vite. Oh. Elles sont prises, Victorina ? Oui, papa. Tes épaules tombent, Victorina ? Un peu, maman. L'éclat de pelle tremble, puis tient. Papa s'accroupit à la même hauteur, sans parler. Je suis déçue. Tu as une boule, Victorina ? Oui, papa. Ses épaules restent basses, près des chaînes. Elle tourne la tête vers le bac.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Ava arrive au parc avec papa. Les balançoires sont prises. Ava sent une boule. Elle dit : je suis &lt;emphasis&gt;déçu&lt;/emphasis&gt;e. Papa écoute. Papa dit : un souhait peut attendre. On nomme. On cherche une autre idée. Ava souffle. Elle dit : le bac à sable. C'est une autre idée. Ils vont au bac. Ava creuse. La déception diminue. [pause]</t>
+          <t>Victorina connaît le parc, ses odeurs, ses bruits. Je le connais, papa. Tu le connais, le parc ? Oui, papa. Les aiguilles de pin craquent sous les chaussures. Elles craquent, maman. Tu les entends, les aiguilles ? Oui, maman. Ça sent le pin, un peu tiède. Ça sent le pin. Tu le sens, le pin ? Oui, papa. Une pelle rouge attend près du bac. Elle est rouge ! Tu la vois, la pelle ? Oui, maman. Sur le manche, un &lt;emphasis&gt;éclat de pelle&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Un seau jaune repose contre le sable. Le seau est jaune. Il attend, près du bac. Oui. Les chaînes des balançoires cliquettent, plus loin. Je les entends. Elles bougent, Victorina ? Oui, maman. Un détail paraît nouveau, sur le manche. Le point clair. Tu le regardes, Victorina ? Oui, papa. En ce moment, Victorina veut la balançoire. Je veux celle-là, maintenant ! Tout de suite ? Oui, papa. Victorina court trop vite vers les chaînes. Les deux balançoires bougent, occupées. Il n'y a plus de place. Elles sont prises. Le sourire de Victorina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Sa poitrine va trop vite. Oh. Elles sont prises, Victorina ? Oui, papa. Tes épaules tombent, Victorina ? Un peu, maman. L'éclat de pelle tremble, puis tient. Papa s'accroupit à la même hauteur, sans parler. Je suis déçue. Tu as une boule, Victorina ? Oui, papa. Ses épaules restent basses, près des chaînes. Elle tourne la tête vers le bac. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>déçu</t>
+          <t>éclat de pelle</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,54 +1321,68 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=élan puis déception; intensite=2; destinataire=enfant; sous_texte=elle_veut_la_balancoire_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Des aiguilles de pin sont sur le chemin.
-narrateur|Elles piquent un peu sous les chaussures.
-narrateur|Un seau jaune attend près du sable.
-narrateur|Une sonnette de vélo tinte, plus loin.
-narrateur|Le toboggan est froid sous la main.
-narrateur|Ça sent le pin, tout doux.
-maman|Je range le sac près des pins.
-papa|On reste ensemble, d'accord ?
-enfant-f|D'accord, papa.
-maman|Tu as vu le seau jaune ?
-enfant-f|Oui. Il attend.
+          <t>narrateur|Victorina connaît le parc, ses odeurs, ses bruits.
+enfant-f|Je le connais, papa.
+papa|Tu le connais, le parc ?
+enfant-f|Oui, papa.
+narrateur|Les aiguilles de pin craquent sous les chaussures.
+enfant-f|Elles craquent, maman.
+maman|Tu les entends, les aiguilles ?
+enfant-f|Oui, maman.
+narrateur|Ça sent le pin, un peu tiède.
+enfant-f|Ça sent le pin.
+papa|Tu le sens, le pin ?
+enfant-f|Oui, papa.
+narrateur|Une pelle rouge attend près du bac.
+enfant-f|Elle est rouge !
+maman|Tu la vois, la pelle ?
+enfant-f|Oui, maman.
+narrateur|Sur le manche, un éclat de pelle luit.
+enfant-f|Il brille, maman.
+maman|Tu le vois, le petit point ?
+enfant-f|Oui, un petit point.
+narrateur|Un seau jaune repose contre le sable.
+enfant-f|Le seau est jaune.
+papa|Il attend, près du bac.
+enfant-f|Oui.
+narrateur|Les chaînes des balançoires cliquettent, plus loin.
+enfant-f|Je les entends.
+maman|Elles bougent, Victorina ?
+enfant-f|Oui, maman.
+narrateur|Un détail paraît nouveau, sur le manche.
+enfant-f|Le point clair.
+papa|Tu le regardes, Victorina ?
+enfant-f|Oui, papa.
 narrateur|En ce moment, Victorina veut la balançoire.
-narrateur|La chaîne brille un peu.
-enfant-f|Celle-là, papa.
-papa|On regarde, oui.
-narrateur|Les deux balançoires bougent déjà.
+enfant-f|Je veux celle-là, maintenant !
+papa|Tout de suite ?
+enfant-f|Oui, papa.
+narrateur|Victorina court trop vite vers les chaînes.
+narrateur|Les deux balançoires bougent, occupées.
 narrateur|Il n'y a plus de place.
-enfant-f|Elles sont prises...
-narrateur|Victorina sent une boule.
-narrateur|Ses épaules tombent un peu.
+enfant-f|Elles sont prises.
+narrateur|Le sourire de Victorina disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Sa poitrine va trop vite.
+enfant-f|Oh.
+papa|Elles sont prises, Victorina ?
+enfant-f|Oui, papa.
+maman|Tes épaules tombent, Victorina ?
+enfant-f|Un peu, maman.
+narrateur|L'éclat de pelle tremble, puis tient.
+narrateur|Papa s'accroupit à la même hauteur, sans parler.
 enfant-f|Je suis déçue.
-papa|Tu es déçue. Ce n'est pas honteux.
-papa|Un souhait peut attendre.
-papa|On nomme. On cherche une autre idée.
-maman|Souffle une fois, Victorina.
-narrateur|Victorina souffle.
-narrateur|Elle regarde le seau jaune.
-enfant-f|Le bac à sable, alors.
-papa|Le bac. C'est une autre idée.
-maman|Bravo. Tu as nommé : déçue.
-narrateur|Ils vont au bac.
-narrateur|Le sable est frais et un peu lourd.
-narrateur|Victorina creuse.
-narrateur|Le seau jaune se remplit.
-enfant-f|Un tas, papa.
-papa|Un tas, oui.
-maman|Tu veux un autre seau ?
-enfant-f|Celui-là. Le jaune.
-narrateur|La déception diminue.
-papa|Être déçue, ce n'est pas honteux.
-papa|Une autre idée peut venir.
-enfant-f|Le bac, alors.
-maman|Oui. Le bac.
-narrateur|Les aiguilles de pin restent sur le chemin.
-narrateur|La sonnette tinte encore, plus loin.</t>
+papa|Tu as une boule, Victorina ?
+enfant-f|Oui, papa.
+narrateur|Ses épaules restent basses, près des chaînes.
+narrateur|Elle tourne la tête vers le bac.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1405,12 +1419,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Les balançoires sont prises. Quelle émotion ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Les &lt;emphasis level="moderate"&gt;balançoires&lt;/emphasis&gt; sont prises. Quelle émotion ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Les balançoires sont prises. Quelle émotion ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Les &lt;emphasis&gt;balançoires&lt;/emphasis&gt; sont prises. Quelle émotion ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1473,7 +1487,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1484,7 +1498,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1499,34 +1513,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>balançoires</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1541,22 +1559,23 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=les_balancoires_sont_prises_quelle_emotion; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Les balançoires sont prises. Quelle émotion ?</t>
+          <t>narrateur|Les balançoires sont prises.
+narrateur|Quelle émotion ?</t>
         </is>
       </c>
     </row>
@@ -1583,17 +1602,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Victorina a du sable sur les doigts. Je suis déçue. Oui. Et tu as trouvé une autre idée. Le souhait peut attendre. Bravo. Tu as dit ce que tu sentais. Tu as choisi le bac ? Oui. Le bac. Le seau jaune est plein. Le sable sent la terre froide.</t>
+          <t>Victorina reste près des chaînes, un instant. Je ne peux pas. Tu regardes où, Victorina ? Le bac. Elle avance trop vite vers le sable. Puis elle s'arrête. Victorina refuse de foncer. Personne ne parle. Elle observe le bac, un instant. Elle écoute le parc, près des aiguilles. Le bac, alors. Tu vas vers le sable ? Oui, maman. Victorina s'agenouille près du bac. Le sable est frais, un peu lourd. Il est froid. Tes mains sont dedans ? Oui, papa. Victorina creuse avec les doigts. Un petit trou s'ouvre, tout près du seau. Un trou, papa. Merci, Victorina. Papa reste à la même hauteur. Le seau jaune est vide, Victorina ? Oui, maman. Elle pousse un peu de sable dans le seau. Il se remplit. Le sable tient, Victorina ? Un peu, papa. Tes doigts sont froids, Victorina ? Un peu, maman. Le ventre de Victorina se desserre. Les épaules se relèvent un peu. Je creuse. On reste près du bac ? Oui. Les aiguilles de pin restent au bord ? Oui, maman. Le trou s'agrandit, sans se presser. Il est à moi. Le sable est lourd, Victorina ? Oui, papa.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Victorina a du sable sur les doigts. Je suis déçue. Oui. Et tu as trouvé une autre idée. Le souhait peut attendre. Bravo. Tu as dit ce que tu sentais. Tu as choisi le bac ? Oui. Le bac. Le seau jaune est plein. Le sable sent la terre froide.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorina reste près des chaînes, un instant. Je ne peux pas. Tu regardes où, Victorina ? Le &lt;emphasis level="moderate"&gt;bac&lt;/emphasis&gt;. Elle avance trop vite vers le sable. Puis elle s'arrête. Victorina refuse de foncer. Personne ne parle. Elle observe le bac, un instant. Elle écoute le parc, près des aiguilles. Le bac, alors. Tu vas vers le sable ? Oui, maman. Victorina s'agenouille près du bac. Le sable est frais, un peu lourd. Il est froid. Tes mains sont dedans ? Oui, papa. Victorina creuse avec les doigts. Un petit trou s'ouvre, tout près du seau. Un trou, papa. Merci, Victorina. Papa reste à la même hauteur. Le seau jaune est vide, Victorina ? Oui, maman. Elle pousse un peu de sable dans le seau. Il se remplit. Le sable tient, Victorina ? Un peu, papa. Tes doigts sont froids, Victorina ? Un peu, maman. Le ventre de Victorina se desserre. Les épaules se relèvent un peu. Je creuse. On reste près du bac ? Oui. Les aiguilles de pin restent au bord ? Oui, maman. Le trou s'agrandit, sans se presser. Il est à moi. Le sable est lourd, Victorina ? Oui, papa.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Ava a dit : je suis &lt;emphasis&gt;déçu&lt;/emphasis&gt;e. Elle a trouvé une autre idée. [pause]</t>
+          <t>Victorina reste près des chaînes, un instant. Je ne peux pas. Tu regardes où, Victorina ? Le &lt;emphasis&gt;bac&lt;/emphasis&gt;. Elle avance trop vite vers le sable. Puis elle s'arrête. Victorina refuse de foncer. Personne ne parle. Elle observe le bac, un instant. Elle écoute le parc, près des aiguilles. Le bac, alors. Tu vas vers le sable ? Oui, maman. Victorina s'agenouille près du bac. Le sable est frais, un peu lourd. Il est froid. Tes mains sont dedans ? Oui, papa. Victorina creuse avec les doigts. Un petit trou s'ouvre, tout près du seau. Un trou, papa. Merci, Victorina. Papa reste à la même hauteur. Le seau jaune est vide, Victorina ? Oui, maman. Elle pousse un peu de sable dans le seau. Il se remplit. Le sable tient, Victorina ? Un peu, papa. Tes doigts sont froids, Victorina ? Un peu, maman. Le ventre de Victorina se desserre. Les épaules se relèvent un peu. Je creuse. On reste près du bac ? Oui. Les aiguilles de pin restent au bord ? Oui, maman. Le trou s'agrandit, sans se presser. Il est à moi. Le sable est lourd, Victorina ? Oui, papa. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1640,7 +1659,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1648,10 +1667,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1674,30 +1693,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>déçu</t>
+          <t>bac</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1706,10 +1725,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1722,20 +1741,53 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis souffle_plus_large; intensite=2; destinataire=enfant; sous_texte=elle_nomme_puis_elle_creuse_au_bac; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Victorina a du sable sur les doigts.
-enfant-f|Je suis déçue.
-papa|Oui. Et tu as trouvé une autre idée.
-maman|Le souhait peut attendre.
-papa|Bravo. Tu as dit ce que tu sentais.
-papa|Tu as choisi le bac ?
-enfant-f|Oui. Le bac.
-narrateur|Le seau jaune est plein.
-narrateur|Le sable sent la terre froide.</t>
+          <t>narrateur|Victorina reste près des chaînes, un instant.
+enfant-f|Je ne peux pas.
+papa|Tu regardes où, Victorina ?
+enfant-f|Le bac.
+narrateur|Elle avance trop vite vers le sable.
+narrateur|Puis elle s'arrête.
+narrateur|Victorina refuse de foncer.
+narrateur|Personne ne parle.
+narrateur|Elle observe le bac, un instant.
+narrateur|Elle écoute le parc, près des aiguilles.
+enfant-f|Le bac, alors.
+maman|Tu vas vers le sable ?
+enfant-f|Oui, maman.
+narrateur|Victorina s'agenouille près du bac.
+narrateur|Le sable est frais, un peu lourd.
+enfant-f|Il est froid.
+papa|Tes mains sont dedans ?
+enfant-f|Oui, papa.
+narrateur|Victorina creuse avec les doigts.
+narrateur|Un petit trou s'ouvre, tout près du seau.
+enfant-f|Un trou, papa.
+papa|Merci, Victorina.
+narrateur|Papa reste à la même hauteur.
+maman|Le seau jaune est vide, Victorina ?
+enfant-f|Oui, maman.
+narrateur|Elle pousse un peu de sable dans le seau.
+enfant-f|Il se remplit.
+papa|Le sable tient, Victorina ?
+enfant-f|Un peu, papa.
+maman|Tes doigts sont froids, Victorina ?
+enfant-f|Un peu, maman.
+narrateur|Le ventre de Victorina se desserre.
+narrateur|Les épaules se relèvent un peu.
+enfant-f|Je creuse.
+papa|On reste près du bac ?
+enfant-f|Oui.
+maman|Les aiguilles de pin restent au bord ?
+enfant-f|Oui, maman.
+narrateur|Le trou s'agrandit, sans se presser.
+enfant-f|Il est à moi.
+papa|Le sable est lourd, Victorina ?
+enfant-f|Oui, papa.</t>
         </is>
       </c>
     </row>
@@ -1762,17 +1814,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Papa essuie le seau. Le plastique est un peu mouillé. Tu donnes la main ? Oui. Ta main. Tu as trouvé une autre idée. Je suis moins déçue. Le bac a aidé. Victorina donne la main. Ils quittent le chemin de pin.</t>
+          <t>Des aiguilles de pin occupent le bac. Le bac est plein ! Victorina veut la pelle, tout de suite. Le manche ne bouge pas. Elle est coincée ! La lame reste sous le sable lourd. Victorina tire trop vite sur le manche. La pelle reste coincée, au fond. Elle ne vient pas. Victorina avance les mains, trop vite. Puis elle s'arrête net. Victorina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la pelle, un instant. Elle écoute le parc, près du bac et du sable. Sur le manche, un éclat de pelle luit. Là, sur le manche. Tu vois le point, Victorina ? Oui, papa. Victorina écarte les aiguilles, sans se presser. Le sable autour de la lame s'ouvre. Un peu, papa. La lame bouge, Victorina ? Un peu, maman. Elle creuse autour, tout près de la lame. La pelle se libère, presque. Elle vient ! Tu la tiens, Victorina ? Oui, papa. Le trou a failli se refermer. Victorina pose la pelle, sans se presser. Poumf. Le sable est lourd, Victorina ? Oui, maman. Elle creuse un vrai trou, plus large. Le seau se remplit, Victorina ? Oui, papa. Tes genoux sont froids, Victorina ? Un peu, maman. Le trou tient, au bord du bac. Il tient. On reste ici, Victorina ? Oui.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Papa essuie le seau. Le plastique est un peu mouillé. Tu donnes la main ? Oui. Ta main. Tu as trouvé une autre idée. Je suis moins déçue. Le bac a aidé. Victorina donne la main. Ils quittent le chemin de pin.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Des aiguilles de pin occupent le bac. Le bac est plein ! Victorina veut la pelle, tout de suite. Le manche ne bouge pas. Elle est coincée ! La lame reste sous le sable lourd. Victorina tire trop vite sur le manche. La pelle reste coincée, au fond. Elle ne vient pas. Victorina avance les mains, trop vite. Puis elle s'arrête net. Victorina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la pelle, un instant. Elle écoute le parc, près du bac et du sable. Sur le manche, un &lt;emphasis level="moderate"&gt;éclat de pelle&lt;/emphasis&gt; luit. Là, sur le manche. Tu vois le point, Victorina ? Oui, papa. Victorina écarte les aiguilles, sans se presser. Le sable autour de la lame s'ouvre. Un peu, papa. La lame bouge, Victorina ? Un peu, maman. Elle creuse autour, tout près de la lame. La pelle se libère, presque. Elle vient ! Tu la tiens, Victorina ? Oui, papa. Le trou a failli se refermer. Victorina pose la pelle, sans se presser. Poumf. Le sable est lourd, Victorina ? Oui, maman. Elle creuse un vrai trou, plus large. Le seau se remplit, Victorina ? Oui, papa. Tes genoux sont froids, Victorina ? Un peu, maman. Le trou tient, au bord du bac. Il tient. On reste ici, Victorina ? Oui.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Papa essuie le seau. Ava donne la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Des aiguilles de pin occupent le bac. Le bac est plein ! Victorina veut la pelle, tout de suite. Le manche ne bouge pas. Elle est coincée ! La lame reste sous le sable lourd. Victorina tire trop vite sur le manche. La pelle reste coincée, au fond. Elle ne vient pas. Victorina avance les mains, trop vite. Puis elle s'arrête net. Victorina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la pelle, un instant. Elle écoute le parc, près du bac et du sable. Sur le manche, un &lt;emphasis&gt;éclat de pelle&lt;/emphasis&gt; luit. Là, sur le manche. Tu vois le point, Victorina ? Oui, papa. Victorina écarte les aiguilles, sans se presser. Le sable autour de la lame s'ouvre. Un peu, papa. La lame bouge, Victorina ? Un peu, maman. Elle creuse autour, tout près de la lame. La pelle se libère, presque. Elle vient ! Tu la tiens, Victorina ? Oui, papa. Le trou a failli se refermer. Victorina pose la pelle, sans se presser. Poumf. Le sable est lourd, Victorina ? Oui, maman. Elle creuse un vrai trou, plus large. Le seau se remplit, Victorina ? Oui, papa. Tes genoux sont froids, Victorina ? Un peu, maman. Le trou tient, au bord du bac. Il tient. On reste ici, Victorina ? Oui. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1819,7 +1871,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1827,10 +1879,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.18</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1853,30 +1905,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de pelle</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1885,10 +1937,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1899,18 +1951,57 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=bac_occupe_pelle_coincee_elle_refuse_de_foncer; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Papa essuie le seau.
-narrateur|Le plastique est un peu mouillé.
-maman|Tu donnes la main ?
-enfant-f|Oui. Ta main.
-papa|Tu as trouvé une autre idée.
-enfant-f|Je suis moins déçue.
-maman|Le bac a aidé.
-narrateur|Victorina donne la main.
-narrateur|Ils quittent le chemin de pin.</t>
+          <t>narrateur|Des aiguilles de pin occupent le bac.
+enfant-f|Le bac est plein !
+narrateur|Victorina veut la pelle, tout de suite.
+narrateur|Le manche ne bouge pas.
+enfant-f|Elle est coincée !
+narrateur|La lame reste sous le sable lourd.
+narrateur|Victorina tire trop vite sur le manche.
+narrateur|La pelle reste coincée, au fond.
+enfant-f|Elle ne vient pas.
+narrateur|Victorina avance les mains, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Victorina refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe la pelle, un instant.
+narrateur|Elle écoute le parc, près du bac et du sable.
+narrateur|Sur le manche, un éclat de pelle luit.
+enfant-f|Là, sur le manche.
+papa|Tu vois le point, Victorina ?
+enfant-f|Oui, papa.
+narrateur|Victorina écarte les aiguilles, sans se presser.
+narrateur|Le sable autour de la lame s'ouvre.
+enfant-f|Un peu, papa.
+maman|La lame bouge, Victorina ?
+enfant-f|Un peu, maman.
+narrateur|Elle creuse autour, tout près de la lame.
+narrateur|La pelle se libère, presque.
+enfant-f|Elle vient !
+papa|Tu la tiens, Victorina ?
+enfant-f|Oui, papa.
+narrateur|Le trou a failli se refermer.
+narrateur|Victorina pose la pelle, sans se presser.
+enfant-f|Poumf.
+maman|Le sable est lourd, Victorina ?
+enfant-f|Oui, maman.
+narrateur|Elle creuse un vrai trou, plus large.
+papa|Le seau se remplit, Victorina ?
+enfant-f|Oui, papa.
+maman|Tes genoux sont froids, Victorina ?
+enfant-f|Un peu, maman.
+narrateur|Le trou tient, au bord du bac.
+enfant-f|Il tient.
+papa|On reste ici, Victorina ?
+enfant-f|Oui.</t>
         </is>
       </c>
     </row>
@@ -1937,17 +2028,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis déçue. J'ai trouvé une autre idée. Un souhait peut attendre. Bravo, Victorina.</t>
+          <t>Ils restent près du bac. Maman essuie un peu de sable. Les balançoires étaient prises, papa. Tu l'as vu, toi ? Oui, près des chaînes. On est bien, ici. Victorina tapote le manche du doigt. Il a une trace de sable. Tu la vois, la trace ? Oui, maman. Le trou est resté, Victorina. Oui, avec le seau. Ça sent le pin, un peu tiède. Et le sable, maman. Oui, dans l'air. Le parc est calme, Victorina ? Oui, papa. La pelle reste près du trou. Un éclat de pelle tient sur le manche.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis déçue. J'ai trouvé une autre idée. Un souhait peut attendre. Bravo, Victorina.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du bac. Maman essuie un peu de sable. Les balançoires étaient prises, papa. Tu l'as vu, toi ? Oui, près des chaînes. On est bien, ici. Victorina tapote le manche du doigt. Il a une trace de sable. Tu la vois, la trace ? Oui, maman. Le trou est resté, Victorina. Oui, avec le seau. Ça sent le pin, un peu tiède. Et le sable, maman. Oui, dans l'air. Le parc est calme, Victorina ? Oui, papa. La pelle reste près du trou. Un &lt;emphasis level="moderate"&gt;éclat de pelle&lt;/emphasis&gt; tient sur le manche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du bac. Maman essuie un peu de sable. Les balançoires étaient prises, papa. Tu l'as vu, toi ? Oui, près des chaînes. On est bien, ici. Victorina tapote le manche du doigt. Il a une trace de sable. Tu la vois, la trace ? Oui, maman. Le trou est resté, Victorina. Oui, avec le seau. Ça sent le pin, un peu tiède. Et le sable, maman. Oui, dans l'air. Le parc est calme, Victorina ? Oui, papa. La pelle reste près du trou. Un &lt;emphasis&gt;éclat de pelle&lt;/emphasis&gt; tient sur le manche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -1994,7 +2085,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2002,10 +2093,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2014,12 +2105,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2028,17 +2119,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de pelle</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2047,11 +2142,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2060,27 +2155,46 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_manche; tempo=très posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai dit : je suis déçue.
-enfant-f|J'ai trouvé une autre idée.
-papa|Un souhait peut attendre.
-maman|Bravo, Victorina.</t>
+          <t>narrateur|Ils restent près du bac.
+narrateur|Maman essuie un peu de sable.
+enfant-f|Les balançoires étaient prises, papa.
+papa|Tu l'as vu, toi ?
+enfant-f|Oui, près des chaînes.
+maman|On est bien, ici.
+narrateur|Victorina tapote le manche du doigt.
+enfant-f|Il a une trace de sable.
+maman|Tu la vois, la trace ?
+enfant-f|Oui, maman.
+papa|Le trou est resté, Victorina.
+enfant-f|Oui, avec le seau.
+narrateur|Ça sent le pin, un peu tiède.
+enfant-f|Et le sable, maman.
+maman|Oui, dans l'air.
+papa|Le parc est calme, Victorina ?
+enfant-f|Oui, papa.
+narrateur|La pelle reste près du trou.
+narrateur|Un éclat de pelle tient sur le manche.</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2151,6 +2265,13 @@
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>